<commit_message>
Add production logfile workflow for Microtom
</commit_message>
<xml_diff>
--- a/master_data/Parameterliste SAR41-MAS-004_V11.11.25.xlsx
+++ b/master_data/Parameterliste SAR41-MAS-004_V11.11.25.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="25080" yWindow="-120" windowWidth="25440" windowHeight="15270" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Parameter" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameter" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="rng_Lieferanten">#REF!</definedName>
@@ -117,7 +117,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -275,6 +275,21 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -736,7 +751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S742"/>
+  <dimension ref="A1:S744"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="16.140625" bestFit="1" customWidth="1" style="3" min="1" max="1"/>
@@ -47371,416 +47386,399 @@
       <c r="P691" s="9" t="n"/>
     </row>
     <row r="692">
-      <c r="A692" s="19" t="n"/>
-      <c r="B692" s="20" t="n"/>
-      <c r="C692" s="44" t="n"/>
-      <c r="D692" s="47" t="n"/>
-      <c r="H692" s="53" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="J692" s="21" t="n"/>
-      <c r="K692" s="53" t="n"/>
-      <c r="M692" s="9" t="n"/>
-      <c r="N692" s="9" t="n"/>
-      <c r="O692" s="9" t="n"/>
-      <c r="P692" s="9" t="n"/>
+      <c r="A692" s="58" t="inlineStr">
+        <is>
+          <t>MAS</t>
+        </is>
+      </c>
+      <c r="B692" s="62" t="inlineStr">
+        <is>
+          <t>0029</t>
+        </is>
+      </c>
+      <c r="C692" s="63" t="n"/>
+      <c r="D692" s="64" t="n"/>
+      <c r="E692" s="58" t="inlineStr"/>
+      <c r="F692" s="58" t="inlineStr">
+        <is>
+          <t>String - Write</t>
+        </is>
+      </c>
+      <c r="G692" s="58" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H692" s="58" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="I692" s="58" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="J692" s="55" t="inlineStr">
+        <is>
+          <t>MAS0029 Produktions-Auftrags-ID / Logfile-Name</t>
+        </is>
+      </c>
+      <c r="K692" s="58" t="n"/>
+      <c r="L692" s="58" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="M692" s="65" t="inlineStr">
+        <is>
+          <t>String-ID der aktuellen Produktion. Dieser Wert wird beim Start (MAS0002=1) als Dateinamenszusatz fuer die Produktions-Logfiles verwendet.</t>
+        </is>
+      </c>
+      <c r="N692" s="66" t="n"/>
+      <c r="O692" s="66" t="n"/>
+      <c r="P692" s="66" t="n"/>
+      <c r="Q692" s="53" t="n"/>
+      <c r="R692" s="53" t="n"/>
+      <c r="S692" s="53" t="n"/>
     </row>
     <row r="693">
-      <c r="A693" s="19" t="n"/>
-      <c r="B693" s="20" t="n"/>
-      <c r="C693" s="44" t="n"/>
-      <c r="D693" s="47" t="n"/>
-      <c r="H693" s="53" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="J693" s="21" t="n"/>
-      <c r="K693" s="53" t="n"/>
-      <c r="M693" s="9" t="n"/>
-      <c r="N693" s="9" t="n"/>
-      <c r="O693" s="9" t="n"/>
-      <c r="P693" s="9" t="n"/>
+      <c r="A693" s="58" t="inlineStr">
+        <is>
+          <t>MAS</t>
+        </is>
+      </c>
+      <c r="B693" s="62" t="inlineStr">
+        <is>
+          <t>0030</t>
+        </is>
+      </c>
+      <c r="C693" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="D693" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="E693" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="F693" s="58" t="inlineStr">
+        <is>
+          <t>Status - Read</t>
+        </is>
+      </c>
+      <c r="G693" s="58" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="H693" s="58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I693" s="58" t="inlineStr">
+        <is>
+          <t>uint8</t>
+        </is>
+      </c>
+      <c r="J693" s="55" t="inlineStr">
+        <is>
+          <t>MAS0030 Produktions-Logfiles abholbereit</t>
+        </is>
+      </c>
+      <c r="K693" s="58" t="n"/>
+      <c r="L693" s="58" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="M693" s="65" t="inlineStr">
+        <is>
+          <t>0 - keine Produktions-Logfiles abholbereit
+1 - Produktions-Logfiles der letzten Produktion sind ueber /api/production/logfiles/* abholbereit</t>
+        </is>
+      </c>
+      <c r="N693" s="66" t="n"/>
+      <c r="O693" s="66" t="n"/>
+      <c r="P693" s="66" t="n"/>
+      <c r="Q693" s="53" t="n"/>
+      <c r="R693" s="53" t="n"/>
+      <c r="S693" s="53" t="n"/>
     </row>
     <row r="694">
-      <c r="A694" s="19" t="inlineStr">
+      <c r="A694" s="19" t="n"/>
+      <c r="B694" s="20" t="n"/>
+      <c r="C694" s="44" t="n"/>
+      <c r="D694" s="47" t="n"/>
+      <c r="H694" s="53" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J694" s="21" t="n"/>
+      <c r="K694" s="53" t="n"/>
+      <c r="M694" s="9" t="n"/>
+      <c r="N694" s="9" t="n"/>
+      <c r="O694" s="9" t="n"/>
+      <c r="P694" s="9" t="n"/>
+    </row>
+    <row r="695">
+      <c r="A695" s="19" t="n"/>
+      <c r="B695" s="20" t="n"/>
+      <c r="C695" s="44" t="n"/>
+      <c r="D695" s="47" t="n"/>
+      <c r="H695" s="53" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J695" s="21" t="n"/>
+      <c r="K695" s="53" t="n"/>
+      <c r="M695" s="9" t="n"/>
+      <c r="N695" s="9" t="n"/>
+      <c r="O695" s="9" t="n"/>
+      <c r="P695" s="9" t="n"/>
+    </row>
+    <row r="696">
+      <c r="A696" s="19" t="inlineStr">
         <is>
           <t>MAW</t>
         </is>
       </c>
-      <c r="B694" s="20" t="inlineStr">
+      <c r="B696" s="20" t="inlineStr">
         <is>
           <t>0001</t>
         </is>
       </c>
-      <c r="C694" s="44" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D694" s="48" t="n">
+      <c r="C696" s="44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D696" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="E694" s="19" t="n">
+      <c r="E696" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="F694" s="19" t="inlineStr">
+      <c r="F696" s="19" t="inlineStr">
         <is>
           <t>OFF/ON</t>
         </is>
       </c>
-      <c r="G694" s="19" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="H694" s="58" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I694" s="19" t="inlineStr">
+      <c r="G696" s="19" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="H696" s="58" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I696" s="19" t="inlineStr">
         <is>
           <t>bool</t>
         </is>
       </c>
-      <c r="J694" s="19" t="inlineStr">
+      <c r="J696" s="19" t="inlineStr">
         <is>
           <t>MAW0001 Warnung Etikettenfüllstand Abwicklung</t>
         </is>
       </c>
-      <c r="K694" s="58" t="n"/>
-      <c r="L694" s="19" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="M694" s="26" t="inlineStr">
+      <c r="K696" s="58" t="n"/>
+      <c r="L696" s="19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="M696" s="26" t="inlineStr">
         <is>
           <t>Der Füllstand der Etiketten Abwickeleinheit ist tiefer als der eingestellte Wert</t>
         </is>
       </c>
-      <c r="N694" s="26" t="n"/>
-      <c r="O694" s="26" t="n"/>
-      <c r="P694" s="26" t="n"/>
-    </row>
-    <row r="695">
-      <c r="A695" s="19" t="inlineStr">
-        <is>
-          <t>MAW</t>
-        </is>
-      </c>
-      <c r="B695" s="20" t="inlineStr">
-        <is>
-          <t>0002</t>
-        </is>
-      </c>
-      <c r="C695" s="44" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D695" s="48" t="n">
-        <v>1</v>
-      </c>
-      <c r="E695" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="F695" s="19" t="inlineStr">
-        <is>
-          <t>OFF/ON</t>
-        </is>
-      </c>
-      <c r="G695" s="19" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="H695" s="58" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I695" s="19" t="inlineStr">
-        <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="J695" s="19" t="inlineStr">
-        <is>
-          <t>MAW0002 Warnung Etikettenfüllstand Aufwicklung</t>
-        </is>
-      </c>
-      <c r="K695" s="58" t="n"/>
-      <c r="L695" s="19" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="M695" s="26" t="inlineStr">
-        <is>
-          <t>Der Füllstand der Etiketten Aufwickeleinheit ist tiefer als der eingestellte Wert</t>
-        </is>
-      </c>
-      <c r="N695" s="26" t="n"/>
-      <c r="O695" s="26" t="n"/>
-      <c r="P695" s="26" t="n"/>
-    </row>
-    <row r="696">
-      <c r="A696" s="19" t="n"/>
-      <c r="B696" s="4" t="n"/>
-      <c r="C696" s="44" t="n"/>
-      <c r="D696" s="48" t="n"/>
-      <c r="E696" s="19" t="n"/>
-      <c r="F696" s="19" t="n"/>
-      <c r="G696" s="19" t="n"/>
-      <c r="H696" s="58" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I696" s="19" t="n"/>
-      <c r="J696" s="19" t="n"/>
-      <c r="K696" s="58" t="n"/>
-      <c r="L696" s="19" t="n"/>
-      <c r="M696" s="26" t="n"/>
       <c r="N696" s="26" t="n"/>
       <c r="O696" s="26" t="n"/>
       <c r="P696" s="26" t="n"/>
     </row>
     <row r="697">
-      <c r="A697" s="19" t="n"/>
-      <c r="B697" s="4" t="n"/>
-      <c r="C697" s="44" t="n"/>
-      <c r="D697" s="48" t="n"/>
-      <c r="E697" s="19" t="n"/>
-      <c r="F697" s="19" t="n"/>
-      <c r="G697" s="19" t="n"/>
+      <c r="A697" s="19" t="inlineStr">
+        <is>
+          <t>MAW</t>
+        </is>
+      </c>
+      <c r="B697" s="20" t="inlineStr">
+        <is>
+          <t>0002</t>
+        </is>
+      </c>
+      <c r="C697" s="44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D697" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="E697" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F697" s="19" t="inlineStr">
+        <is>
+          <t>OFF/ON</t>
+        </is>
+      </c>
+      <c r="G697" s="19" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
       <c r="H697" s="58" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="I697" s="19" t="n"/>
-      <c r="J697" s="19" t="n"/>
+      <c r="I697" s="19" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="J697" s="19" t="inlineStr">
+        <is>
+          <t>MAW0002 Warnung Etikettenfüllstand Aufwicklung</t>
+        </is>
+      </c>
       <c r="K697" s="58" t="n"/>
-      <c r="L697" s="19" t="n"/>
-      <c r="M697" s="26" t="n"/>
+      <c r="L697" s="19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="M697" s="26" t="inlineStr">
+        <is>
+          <t>Der Füllstand der Etiketten Aufwickeleinheit ist tiefer als der eingestellte Wert</t>
+        </is>
+      </c>
       <c r="N697" s="26" t="n"/>
       <c r="O697" s="26" t="n"/>
       <c r="P697" s="26" t="n"/>
     </row>
     <row r="698">
-      <c r="A698" s="19" t="inlineStr">
+      <c r="A698" s="19" t="n"/>
+      <c r="B698" s="4" t="n"/>
+      <c r="C698" s="44" t="n"/>
+      <c r="D698" s="48" t="n"/>
+      <c r="E698" s="19" t="n"/>
+      <c r="F698" s="19" t="n"/>
+      <c r="G698" s="19" t="n"/>
+      <c r="H698" s="58" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I698" s="19" t="n"/>
+      <c r="J698" s="19" t="n"/>
+      <c r="K698" s="58" t="n"/>
+      <c r="L698" s="19" t="n"/>
+      <c r="M698" s="26" t="n"/>
+      <c r="N698" s="26" t="n"/>
+      <c r="O698" s="26" t="n"/>
+      <c r="P698" s="26" t="n"/>
+    </row>
+    <row r="699">
+      <c r="A699" s="19" t="n"/>
+      <c r="B699" s="4" t="n"/>
+      <c r="C699" s="44" t="n"/>
+      <c r="D699" s="48" t="n"/>
+      <c r="E699" s="19" t="n"/>
+      <c r="F699" s="19" t="n"/>
+      <c r="G699" s="19" t="n"/>
+      <c r="H699" s="58" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I699" s="19" t="n"/>
+      <c r="J699" s="19" t="n"/>
+      <c r="K699" s="58" t="n"/>
+      <c r="L699" s="19" t="n"/>
+      <c r="M699" s="26" t="n"/>
+      <c r="N699" s="26" t="n"/>
+      <c r="O699" s="26" t="n"/>
+      <c r="P699" s="26" t="n"/>
+    </row>
+    <row r="700">
+      <c r="A700" s="19" t="inlineStr">
         <is>
           <t>MAE</t>
         </is>
       </c>
-      <c r="B698" s="4" t="inlineStr">
+      <c r="B700" s="4" t="inlineStr">
         <is>
           <t>0001</t>
         </is>
       </c>
-      <c r="C698" s="44" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D698" s="48" t="n">
+      <c r="C700" s="44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D700" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="E698" s="19" t="n">
+      <c r="E700" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="F698" s="19" t="n"/>
-      <c r="G698" s="19" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="H698" s="58" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I698" s="19" t="inlineStr">
+      <c r="F700" s="19" t="n"/>
+      <c r="G700" s="19" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="H700" s="58" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I700" s="19" t="inlineStr">
         <is>
           <t>bool</t>
         </is>
       </c>
-      <c r="J698" s="19" t="inlineStr">
+      <c r="J700" s="19" t="inlineStr">
         <is>
           <t>MAE0001 Not-Aus ausgelöst</t>
         </is>
       </c>
-      <c r="K698" s="58" t="n"/>
-      <c r="L698" s="19" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="M698" s="19" t="inlineStr">
+      <c r="K700" s="58" t="n"/>
+      <c r="L700" s="19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="M700" s="19" t="inlineStr">
         <is>
           <t>Not-Aus wurde betätigt</t>
         </is>
       </c>
-      <c r="N698" s="19" t="inlineStr">
+      <c r="N700" s="19" t="inlineStr">
         <is>
           <t>Not-Aus-Taster gedrückt, Sicherheitskreis unterbrochen</t>
         </is>
       </c>
-      <c r="O698" s="19" t="inlineStr">
+      <c r="O700" s="19" t="inlineStr">
         <is>
           <t>Produktionsstopp</t>
         </is>
       </c>
-      <c r="P698" s="49" t="inlineStr">
+      <c r="P700" s="49" t="inlineStr">
         <is>
           <t>Not-Aus entriegeln, Sicherheitskreis prüfen, 
 Produktion neu starten</t>
         </is>
       </c>
     </row>
-    <row r="699">
-      <c r="A699" s="19" t="inlineStr">
-        <is>
-          <t>MAE</t>
-        </is>
-      </c>
-      <c r="B699" s="4" t="inlineStr">
-        <is>
-          <t>0002</t>
-        </is>
-      </c>
-      <c r="C699" s="44" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D699" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="E699" t="n">
-        <v>0</v>
-      </c>
-      <c r="G699" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="H699" s="53" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I699" t="inlineStr">
-        <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="J699" t="inlineStr">
-        <is>
-          <t>MAE0002 Lichtgitter ausgelöst</t>
-        </is>
-      </c>
-      <c r="K699" s="53" t="n"/>
-      <c r="L699" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="M699" t="inlineStr">
-        <is>
-          <t>Lichtgitter unterbrochen</t>
-        </is>
-      </c>
-      <c r="N699" t="inlineStr">
-        <is>
-          <t>Person oder Objekt im Schutzbereich</t>
-        </is>
-      </c>
-      <c r="O699" t="inlineStr">
-        <is>
-          <t>Produktionspause</t>
-        </is>
-      </c>
-      <c r="P699" t="inlineStr">
-        <is>
-          <t>Schutzbereich freimachen, Start drücken</t>
-        </is>
-      </c>
-    </row>
-    <row r="700">
-      <c r="A700" s="19" t="inlineStr">
-        <is>
-          <t>MAE</t>
-        </is>
-      </c>
-      <c r="B700" s="4" t="inlineStr">
-        <is>
-          <t>0003</t>
-        </is>
-      </c>
-      <c r="C700" s="44" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D700" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="E700" t="n">
-        <v>0</v>
-      </c>
-      <c r="G700" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="H700" s="53" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I700" t="inlineStr">
-        <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="J700" t="inlineStr">
-        <is>
-          <t>MAE0003 Laserschutzgehäuse offen</t>
-        </is>
-      </c>
-      <c r="K700" s="53" t="n"/>
-      <c r="L700" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="M700" t="inlineStr">
-        <is>
-          <t>Laserschutzgehäuse offen</t>
-        </is>
-      </c>
-      <c r="N700" t="inlineStr">
-        <is>
-          <t>Schutzschalter geöffnet</t>
-        </is>
-      </c>
-      <c r="O700" t="inlineStr">
-        <is>
-          <t>Produktionspause</t>
-        </is>
-      </c>
-      <c r="P700" t="inlineStr">
-        <is>
-          <t>Sensorposition prüfen</t>
-        </is>
-      </c>
-    </row>
     <row r="701">
       <c r="A701" s="19" t="inlineStr">
         <is>
@@ -47789,7 +47787,7 @@
       </c>
       <c r="B701" s="4" t="inlineStr">
         <is>
-          <t>0004</t>
+          <t>0002</t>
         </is>
       </c>
       <c r="C701" s="44" t="inlineStr">
@@ -47820,7 +47818,7 @@
       </c>
       <c r="J701" t="inlineStr">
         <is>
-          <t>MAE0004 Störung Portalachsenmotor X</t>
+          <t>MAE0002 Lichtgitter ausgelöst</t>
         </is>
       </c>
       <c r="K701" s="53" t="n"/>
@@ -47831,22 +47829,22 @@
       </c>
       <c r="M701" t="inlineStr">
         <is>
-          <t>Störung Motor X-Achse</t>
+          <t>Lichtgitter unterbrochen</t>
         </is>
       </c>
       <c r="N701" t="inlineStr">
         <is>
-          <t>Überlast oder Blockade</t>
+          <t>Person oder Objekt im Schutzbereich</t>
         </is>
       </c>
       <c r="O701" t="inlineStr">
         <is>
-          <t>Positionierung nicht möglich</t>
+          <t>Produktionspause</t>
         </is>
       </c>
       <c r="P701" t="inlineStr">
         <is>
-          <t>Mechanik und Motor prüfen</t>
+          <t>Schutzbereich freimachen, Start drücken</t>
         </is>
       </c>
     </row>
@@ -47858,7 +47856,7 @@
       </c>
       <c r="B702" s="4" t="inlineStr">
         <is>
-          <t>0005</t>
+          <t>0003</t>
         </is>
       </c>
       <c r="C702" s="44" t="inlineStr">
@@ -47889,7 +47887,7 @@
       </c>
       <c r="J702" t="inlineStr">
         <is>
-          <t>MAE0005 Störung Portalachsenmotor Z</t>
+          <t>MAE0003 Laserschutzgehäuse offen</t>
         </is>
       </c>
       <c r="K702" s="53" t="n"/>
@@ -47900,22 +47898,22 @@
       </c>
       <c r="M702" t="inlineStr">
         <is>
-          <t>Störung Motor Z-Achse</t>
+          <t>Laserschutzgehäuse offen</t>
         </is>
       </c>
       <c r="N702" t="inlineStr">
         <is>
-          <t>Überlast oder Blockade</t>
+          <t>Schutzschalter geöffnet</t>
         </is>
       </c>
       <c r="O702" t="inlineStr">
         <is>
-          <t>Positionierung nicht möglich</t>
+          <t>Produktionspause</t>
         </is>
       </c>
       <c r="P702" t="inlineStr">
         <is>
-          <t>Mechanik und Motor prüfen</t>
+          <t>Sensorposition prüfen</t>
         </is>
       </c>
     </row>
@@ -47927,7 +47925,7 @@
       </c>
       <c r="B703" s="4" t="inlineStr">
         <is>
-          <t>0006</t>
+          <t>0004</t>
         </is>
       </c>
       <c r="C703" s="44" t="inlineStr">
@@ -47958,7 +47956,7 @@
       </c>
       <c r="J703" t="inlineStr">
         <is>
-          <t>MAE0006 Störung Positionsantrieb Etiketten Erfassungssensor</t>
+          <t>MAE0004 Störung Portalachsenmotor X</t>
         </is>
       </c>
       <c r="K703" s="53" t="n"/>
@@ -47969,7 +47967,7 @@
       </c>
       <c r="M703" t="inlineStr">
         <is>
-          <t>Positionsantrieb Erfassungssensor gestört</t>
+          <t>Störung Motor X-Achse</t>
         </is>
       </c>
       <c r="N703" t="inlineStr">
@@ -47996,7 +47994,7 @@
       </c>
       <c r="B704" s="4" t="inlineStr">
         <is>
-          <t>0007</t>
+          <t>0005</t>
         </is>
       </c>
       <c r="C704" s="44" t="inlineStr">
@@ -48027,7 +48025,7 @@
       </c>
       <c r="J704" t="inlineStr">
         <is>
-          <t>MAE0007 Störung Positionsantrieb Etiketten Entnahmesensor</t>
+          <t>MAE0005 Störung Portalachsenmotor Z</t>
         </is>
       </c>
       <c r="K704" s="53" t="n"/>
@@ -48038,7 +48036,7 @@
       </c>
       <c r="M704" t="inlineStr">
         <is>
-          <t>Positionsantrieb Entnahmesensor gestört</t>
+          <t>Störung Motor Z-Achse</t>
         </is>
       </c>
       <c r="N704" t="inlineStr">
@@ -48065,7 +48063,7 @@
       </c>
       <c r="B705" s="4" t="inlineStr">
         <is>
-          <t>0008</t>
+          <t>0006</t>
         </is>
       </c>
       <c r="C705" s="44" t="inlineStr">
@@ -48096,7 +48094,7 @@
       </c>
       <c r="J705" t="inlineStr">
         <is>
-          <t>MAE0008 Störung Positionsantrieb Etikettenführung Einlauf</t>
+          <t>MAE0006 Störung Positionsantrieb Etiketten Erfassungssensor</t>
         </is>
       </c>
       <c r="K705" s="53" t="n"/>
@@ -48107,7 +48105,7 @@
       </c>
       <c r="M705" t="inlineStr">
         <is>
-          <t>Etikettenführung Einlauf gestört</t>
+          <t>Positionsantrieb Erfassungssensor gestört</t>
         </is>
       </c>
       <c r="N705" t="inlineStr">
@@ -48134,7 +48132,7 @@
       </c>
       <c r="B706" s="4" t="inlineStr">
         <is>
-          <t>0009</t>
+          <t>0007</t>
         </is>
       </c>
       <c r="C706" s="44" t="inlineStr">
@@ -48165,7 +48163,7 @@
       </c>
       <c r="J706" t="inlineStr">
         <is>
-          <t>MAE0009 Störung Positionsantrieb Etikettenführung Auslauf</t>
+          <t>MAE0007 Störung Positionsantrieb Etiketten Entnahmesensor</t>
         </is>
       </c>
       <c r="K706" s="53" t="n"/>
@@ -48176,7 +48174,7 @@
       </c>
       <c r="M706" t="inlineStr">
         <is>
-          <t>Etikettenführung Auslauf gestört</t>
+          <t>Positionsantrieb Entnahmesensor gestört</t>
         </is>
       </c>
       <c r="N706" t="inlineStr">
@@ -48203,7 +48201,7 @@
       </c>
       <c r="B707" s="4" t="inlineStr">
         <is>
-          <t>0010</t>
+          <t>0008</t>
         </is>
       </c>
       <c r="C707" s="44" t="inlineStr">
@@ -48234,7 +48232,7 @@
       </c>
       <c r="J707" t="inlineStr">
         <is>
-          <t>MAE0010 Störung Positionsantrieb Material Kontrollkamera</t>
+          <t>MAE0008 Störung Positionsantrieb Etikettenführung Einlauf</t>
         </is>
       </c>
       <c r="K707" s="53" t="n"/>
@@ -48245,7 +48243,7 @@
       </c>
       <c r="M707" t="inlineStr">
         <is>
-          <t>Materialkontrollkamera Positionsantrieb meldet Störung</t>
+          <t>Etikettenführung Einlauf gestört</t>
         </is>
       </c>
       <c r="N707" t="inlineStr">
@@ -48272,7 +48270,7 @@
       </c>
       <c r="B708" s="4" t="inlineStr">
         <is>
-          <t>0011</t>
+          <t>0009</t>
         </is>
       </c>
       <c r="C708" s="44" t="inlineStr">
@@ -48303,7 +48301,7 @@
       </c>
       <c r="J708" t="inlineStr">
         <is>
-          <t>MAE0011 Störung Antriebsmotor Abwicklung</t>
+          <t>MAE0009 Störung Positionsantrieb Etikettenführung Auslauf</t>
         </is>
       </c>
       <c r="K708" s="53" t="n"/>
@@ -48314,7 +48312,7 @@
       </c>
       <c r="M708" t="inlineStr">
         <is>
-          <t>Abwicklungsmotor meldet Störung</t>
+          <t>Etikettenführung Auslauf gestört</t>
         </is>
       </c>
       <c r="N708" t="inlineStr">
@@ -48324,7 +48322,7 @@
       </c>
       <c r="O708" t="inlineStr">
         <is>
-          <t>Produktionspause</t>
+          <t>Positionierung nicht möglich</t>
         </is>
       </c>
       <c r="P708" t="inlineStr">
@@ -48341,7 +48339,7 @@
       </c>
       <c r="B709" s="4" t="inlineStr">
         <is>
-          <t>0012</t>
+          <t>0010</t>
         </is>
       </c>
       <c r="C709" s="44" t="inlineStr">
@@ -48372,7 +48370,7 @@
       </c>
       <c r="J709" t="inlineStr">
         <is>
-          <t>MAE0012 Störung Antriebsmotor Aufwicklung</t>
+          <t>MAE0010 Störung Positionsantrieb Material Kontrollkamera</t>
         </is>
       </c>
       <c r="K709" s="53" t="n"/>
@@ -48383,7 +48381,7 @@
       </c>
       <c r="M709" t="inlineStr">
         <is>
-          <t>Aufwicklungsmotor meldet Störung</t>
+          <t>Materialkontrollkamera Positionsantrieb meldet Störung</t>
         </is>
       </c>
       <c r="N709" t="inlineStr">
@@ -48393,7 +48391,7 @@
       </c>
       <c r="O709" t="inlineStr">
         <is>
-          <t>Produktionspause</t>
+          <t>Positionierung nicht möglich</t>
         </is>
       </c>
       <c r="P709" t="inlineStr">
@@ -48410,7 +48408,7 @@
       </c>
       <c r="B710" s="4" t="inlineStr">
         <is>
-          <t>0013</t>
+          <t>0011</t>
         </is>
       </c>
       <c r="C710" s="44" t="inlineStr">
@@ -48441,7 +48439,7 @@
       </c>
       <c r="J710" t="inlineStr">
         <is>
-          <t>MAE0013 Störung Kommunikation mit Mikrotom</t>
+          <t>MAE0011 Störung Antriebsmotor Abwicklung</t>
         </is>
       </c>
       <c r="K710" s="53" t="n"/>
@@ -48452,22 +48450,22 @@
       </c>
       <c r="M710" t="inlineStr">
         <is>
-          <t>Kommunikation Mikrotom gestört</t>
+          <t>Abwicklungsmotor meldet Störung</t>
         </is>
       </c>
       <c r="N710" t="inlineStr">
         <is>
-          <t>Netzwerkfehler</t>
+          <t>Überlast oder Blockade</t>
         </is>
       </c>
       <c r="O710" t="inlineStr">
         <is>
-          <t>Produktionsstopp</t>
+          <t>Produktionspause</t>
         </is>
       </c>
       <c r="P710" t="inlineStr">
         <is>
-          <t>Verbindung prüfen</t>
+          <t>Mechanik und Motor prüfen</t>
         </is>
       </c>
     </row>
@@ -48479,7 +48477,7 @@
       </c>
       <c r="B711" s="4" t="inlineStr">
         <is>
-          <t>0014</t>
+          <t>0012</t>
         </is>
       </c>
       <c r="C711" s="44" t="inlineStr">
@@ -48510,7 +48508,7 @@
       </c>
       <c r="J711" t="inlineStr">
         <is>
-          <t>MAE0014 Störung Kommunikation mit TTO</t>
+          <t>MAE0012 Störung Antriebsmotor Aufwicklung</t>
         </is>
       </c>
       <c r="K711" s="53" t="n"/>
@@ -48521,22 +48519,22 @@
       </c>
       <c r="M711" t="inlineStr">
         <is>
-          <t>Kommunikation mit TTO gestört</t>
+          <t>Aufwicklungsmotor meldet Störung</t>
         </is>
       </c>
       <c r="N711" t="inlineStr">
         <is>
-          <t>Netzwerkfehler</t>
+          <t>Überlast oder Blockade</t>
         </is>
       </c>
       <c r="O711" t="inlineStr">
         <is>
-          <t>Druck nicht möglich</t>
+          <t>Produktionspause</t>
         </is>
       </c>
       <c r="P711" t="inlineStr">
         <is>
-          <t>TTO prüfen</t>
+          <t>Mechanik und Motor prüfen</t>
         </is>
       </c>
     </row>
@@ -48548,7 +48546,7 @@
       </c>
       <c r="B712" s="4" t="inlineStr">
         <is>
-          <t>0015</t>
+          <t>0013</t>
         </is>
       </c>
       <c r="C712" s="44" t="inlineStr">
@@ -48579,7 +48577,7 @@
       </c>
       <c r="J712" t="inlineStr">
         <is>
-          <t>MAE0015 Störung Kommunikation mit LASER</t>
+          <t>MAE0013 Störung Kommunikation mit Mikrotom</t>
         </is>
       </c>
       <c r="K712" s="53" t="n"/>
@@ -48590,7 +48588,7 @@
       </c>
       <c r="M712" t="inlineStr">
         <is>
-          <t>Kommunikation mit Laser gestört</t>
+          <t>Kommunikation Mikrotom gestört</t>
         </is>
       </c>
       <c r="N712" t="inlineStr">
@@ -48600,12 +48598,12 @@
       </c>
       <c r="O712" t="inlineStr">
         <is>
-          <t>Laserbetrieb gestoppt</t>
+          <t>Produktionsstopp</t>
         </is>
       </c>
       <c r="P712" t="inlineStr">
         <is>
-          <t>Laser prüfen</t>
+          <t>Verbindung prüfen</t>
         </is>
       </c>
     </row>
@@ -48617,7 +48615,7 @@
       </c>
       <c r="B713" s="4" t="inlineStr">
         <is>
-          <t>0016</t>
+          <t>0014</t>
         </is>
       </c>
       <c r="C713" s="44" t="inlineStr">
@@ -48648,7 +48646,7 @@
       </c>
       <c r="J713" t="inlineStr">
         <is>
-          <t>MAE0016 Störung Kommunikation mit Abwicklung</t>
+          <t>MAE0014 Störung Kommunikation mit TTO</t>
         </is>
       </c>
       <c r="K713" s="53" t="n"/>
@@ -48659,7 +48657,7 @@
       </c>
       <c r="M713" t="inlineStr">
         <is>
-          <t>Kommunikation mit Abwicklung gestört</t>
+          <t>Kommunikation mit TTO gestört</t>
         </is>
       </c>
       <c r="N713" t="inlineStr">
@@ -48669,12 +48667,12 @@
       </c>
       <c r="O713" t="inlineStr">
         <is>
-          <t>Produktionsstopp</t>
+          <t>Druck nicht möglich</t>
         </is>
       </c>
       <c r="P713" t="inlineStr">
         <is>
-          <t>Verbindung prüfen</t>
+          <t>TTO prüfen</t>
         </is>
       </c>
     </row>
@@ -48686,7 +48684,7 @@
       </c>
       <c r="B714" s="4" t="inlineStr">
         <is>
-          <t>0017</t>
+          <t>0015</t>
         </is>
       </c>
       <c r="C714" s="44" t="inlineStr">
@@ -48717,7 +48715,7 @@
       </c>
       <c r="J714" t="inlineStr">
         <is>
-          <t>MAE0017 Störung Kommunikation mit Aufwicklung</t>
+          <t>MAE0015 Störung Kommunikation mit LASER</t>
         </is>
       </c>
       <c r="K714" s="53" t="n"/>
@@ -48728,7 +48726,7 @@
       </c>
       <c r="M714" t="inlineStr">
         <is>
-          <t>Kommunikation mit Aufwicklung gestört</t>
+          <t>Kommunikation mit Laser gestört</t>
         </is>
       </c>
       <c r="N714" t="inlineStr">
@@ -48738,12 +48736,12 @@
       </c>
       <c r="O714" t="inlineStr">
         <is>
-          <t>Produktionsstopp</t>
+          <t>Laserbetrieb gestoppt</t>
         </is>
       </c>
       <c r="P714" t="inlineStr">
         <is>
-          <t>Verbindung prüfen</t>
+          <t>Laser prüfen</t>
         </is>
       </c>
     </row>
@@ -48755,7 +48753,7 @@
       </c>
       <c r="B715" s="4" t="inlineStr">
         <is>
-          <t>0018</t>
+          <t>0016</t>
         </is>
       </c>
       <c r="C715" s="44" t="inlineStr">
@@ -48786,7 +48784,7 @@
       </c>
       <c r="J715" t="inlineStr">
         <is>
-          <t>MAE0018 Störung Modbus-RTU</t>
+          <t>MAE0016 Störung Kommunikation mit Abwicklung</t>
         </is>
       </c>
       <c r="K715" s="53" t="n"/>
@@ -48797,17 +48795,17 @@
       </c>
       <c r="M715" t="inlineStr">
         <is>
-          <t>Modbus-RTU Fehler</t>
+          <t>Kommunikation mit Abwicklung gestört</t>
         </is>
       </c>
       <c r="N715" t="inlineStr">
         <is>
-          <t>Busunterbruch</t>
+          <t>Netzwerkfehler</t>
         </is>
       </c>
       <c r="O715" t="inlineStr">
         <is>
-          <t>Mehrere Komponenten ohne Funktion</t>
+          <t>Produktionsstopp</t>
         </is>
       </c>
       <c r="P715" t="inlineStr">
@@ -48824,7 +48822,7 @@
       </c>
       <c r="B716" s="4" t="inlineStr">
         <is>
-          <t>0019</t>
+          <t>0017</t>
         </is>
       </c>
       <c r="C716" s="44" t="inlineStr">
@@ -48855,7 +48853,7 @@
       </c>
       <c r="J716" t="inlineStr">
         <is>
-          <t>MAE0019 Störung Encoder Abwicklung</t>
+          <t>MAE0017 Störung Kommunikation mit Aufwicklung</t>
         </is>
       </c>
       <c r="K716" s="53" t="n"/>
@@ -48866,22 +48864,22 @@
       </c>
       <c r="M716" t="inlineStr">
         <is>
-          <t>Encoder Abwicklung fehlerhaft</t>
+          <t>Kommunikation mit Aufwicklung gestört</t>
         </is>
       </c>
       <c r="N716" t="inlineStr">
         <is>
-          <t>Signalverlust oder Blockade</t>
+          <t>Netzwerkfehler</t>
         </is>
       </c>
       <c r="O716" t="inlineStr">
         <is>
-          <t>Produktionspause</t>
+          <t>Produktionsstopp</t>
         </is>
       </c>
       <c r="P716" t="inlineStr">
         <is>
-          <t>Encoder prüfen</t>
+          <t>Verbindung prüfen</t>
         </is>
       </c>
     </row>
@@ -48893,7 +48891,7 @@
       </c>
       <c r="B717" s="4" t="inlineStr">
         <is>
-          <t>0020</t>
+          <t>0018</t>
         </is>
       </c>
       <c r="C717" s="44" t="inlineStr">
@@ -48924,7 +48922,7 @@
       </c>
       <c r="J717" t="inlineStr">
         <is>
-          <t>MAE0020 Störung Encoder Aufwicklung</t>
+          <t>MAE0018 Störung Modbus-RTU</t>
         </is>
       </c>
       <c r="K717" s="53" t="n"/>
@@ -48935,22 +48933,22 @@
       </c>
       <c r="M717" t="inlineStr">
         <is>
-          <t>Encoder Aufwicklung fehlerhaft</t>
+          <t>Modbus-RTU Fehler</t>
         </is>
       </c>
       <c r="N717" t="inlineStr">
         <is>
-          <t>Signalverlust oder Blockade</t>
+          <t>Busunterbruch</t>
         </is>
       </c>
       <c r="O717" t="inlineStr">
         <is>
-          <t>Produktionspause</t>
+          <t>Mehrere Komponenten ohne Funktion</t>
         </is>
       </c>
       <c r="P717" t="inlineStr">
         <is>
-          <t>Encoder prüfen</t>
+          <t>Verbindung prüfen</t>
         </is>
       </c>
     </row>
@@ -48962,7 +48960,7 @@
       </c>
       <c r="B718" s="4" t="inlineStr">
         <is>
-          <t>0021</t>
+          <t>0019</t>
         </is>
       </c>
       <c r="C718" s="44" t="inlineStr">
@@ -48993,7 +48991,7 @@
       </c>
       <c r="J718" t="inlineStr">
         <is>
-          <t>MAE0021 Störung Etiketten Erfassungs-Sensor</t>
+          <t>MAE0019 Störung Encoder Abwicklung</t>
         </is>
       </c>
       <c r="K718" s="53" t="n"/>
@@ -49004,22 +49002,22 @@
       </c>
       <c r="M718" t="inlineStr">
         <is>
-          <t>Etiketten Erfassungs-Sensor gestört</t>
+          <t>Encoder Abwicklung fehlerhaft</t>
         </is>
       </c>
       <c r="N718" t="inlineStr">
         <is>
-          <t>Verschmutzt oder falsch positioniert</t>
+          <t>Signalverlust oder Blockade</t>
         </is>
       </c>
       <c r="O718" t="inlineStr">
         <is>
-          <t>Produktionsstopp</t>
+          <t>Produktionspause</t>
         </is>
       </c>
       <c r="P718" t="inlineStr">
         <is>
-          <t>Sensor reinigen und Positio in Format prüfen</t>
+          <t>Encoder prüfen</t>
         </is>
       </c>
     </row>
@@ -49031,7 +49029,7 @@
       </c>
       <c r="B719" s="4" t="inlineStr">
         <is>
-          <t>0022</t>
+          <t>0020</t>
         </is>
       </c>
       <c r="C719" s="44" t="inlineStr">
@@ -49062,7 +49060,7 @@
       </c>
       <c r="J719" t="inlineStr">
         <is>
-          <t>MAE0022 Störung Etiketten Kontroll-Sensor</t>
+          <t>MAE0020 Störung Encoder Aufwicklung</t>
         </is>
       </c>
       <c r="K719" s="53" t="n"/>
@@ -49073,22 +49071,22 @@
       </c>
       <c r="M719" t="inlineStr">
         <is>
-          <t>Etiketten Kontrollsensor gestört</t>
+          <t>Encoder Aufwicklung fehlerhaft</t>
         </is>
       </c>
       <c r="N719" t="inlineStr">
         <is>
-          <t>Verschmutzt oder falsch positioniert</t>
+          <t>Signalverlust oder Blockade</t>
         </is>
       </c>
       <c r="O719" t="inlineStr">
         <is>
-          <t>Produktionsstopp</t>
+          <t>Produktionspause</t>
         </is>
       </c>
       <c r="P719" t="inlineStr">
         <is>
-          <t>Sensor reinigen und Positio in Format prüfen</t>
+          <t>Encoder prüfen</t>
         </is>
       </c>
     </row>
@@ -49100,7 +49098,7 @@
       </c>
       <c r="B720" s="4" t="inlineStr">
         <is>
-          <t>0023</t>
+          <t>0021</t>
         </is>
       </c>
       <c r="C720" s="44" t="inlineStr">
@@ -49131,7 +49129,7 @@
       </c>
       <c r="J720" t="inlineStr">
         <is>
-          <t>MAE0023 Inkonsistente Bewegung zwischen Auf- und Abwichlung</t>
+          <t>MAE0021 Störung Etiketten Erfassungs-Sensor</t>
         </is>
       </c>
       <c r="K720" s="53" t="n"/>
@@ -49142,161 +49140,161 @@
       </c>
       <c r="M720" t="inlineStr">
         <is>
+          <t>Etiketten Erfassungs-Sensor gestört</t>
+        </is>
+      </c>
+      <c r="N720" t="inlineStr">
+        <is>
+          <t>Verschmutzt oder falsch positioniert</t>
+        </is>
+      </c>
+      <c r="O720" t="inlineStr">
+        <is>
+          <t>Produktionsstopp</t>
+        </is>
+      </c>
+      <c r="P720" t="inlineStr">
+        <is>
+          <t>Sensor reinigen und Positio in Format prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" s="19" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="B721" s="4" t="inlineStr">
+        <is>
+          <t>0022</t>
+        </is>
+      </c>
+      <c r="C721" s="44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D721" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="E721" t="n">
+        <v>0</v>
+      </c>
+      <c r="G721" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="H721" s="53" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I721" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="J721" t="inlineStr">
+        <is>
+          <t>MAE0022 Störung Etiketten Kontroll-Sensor</t>
+        </is>
+      </c>
+      <c r="K721" s="53" t="n"/>
+      <c r="L721" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="M721" t="inlineStr">
+        <is>
+          <t>Etiketten Kontrollsensor gestört</t>
+        </is>
+      </c>
+      <c r="N721" t="inlineStr">
+        <is>
+          <t>Verschmutzt oder falsch positioniert</t>
+        </is>
+      </c>
+      <c r="O721" t="inlineStr">
+        <is>
+          <t>Produktionsstopp</t>
+        </is>
+      </c>
+      <c r="P721" t="inlineStr">
+        <is>
+          <t>Sensor reinigen und Positio in Format prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" s="19" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="B722" s="4" t="inlineStr">
+        <is>
+          <t>0023</t>
+        </is>
+      </c>
+      <c r="C722" s="44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D722" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="E722" t="n">
+        <v>0</v>
+      </c>
+      <c r="G722" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="H722" s="53" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I722" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="J722" t="inlineStr">
+        <is>
+          <t>MAE0023 Inkonsistente Bewegung zwischen Auf- und Abwichlung</t>
+        </is>
+      </c>
+      <c r="K722" s="53" t="n"/>
+      <c r="L722" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="M722" t="inlineStr">
+        <is>
           <t>Inkonsistente Wickelbewegung</t>
         </is>
       </c>
-      <c r="N720" s="12" t="inlineStr">
+      <c r="N722" s="12" t="inlineStr">
         <is>
           <t>Encoderabweichung (Schlupf zwischen Ab und 
 Aufwicklung)</t>
         </is>
       </c>
-      <c r="O720" t="inlineStr">
+      <c r="O722" t="inlineStr">
         <is>
           <t>Produktionspause</t>
         </is>
       </c>
-      <c r="P720" t="inlineStr">
+      <c r="P722" t="inlineStr">
         <is>
           <t>Rollen Reinigen, Format prüfen</t>
-        </is>
-      </c>
-    </row>
-    <row r="721">
-      <c r="A721" s="19" t="inlineStr">
-        <is>
-          <t>MAE</t>
-        </is>
-      </c>
-      <c r="B721" s="4" t="inlineStr">
-        <is>
-          <t>0024</t>
-        </is>
-      </c>
-      <c r="C721" s="44" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D721" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="E721" t="n">
-        <v>0</v>
-      </c>
-      <c r="G721" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="H721" s="53" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I721" t="inlineStr">
-        <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="J721" t="inlineStr">
-        <is>
-          <t>MAE0024 Etikettenbandriss</t>
-        </is>
-      </c>
-      <c r="K721" s="53" t="n"/>
-      <c r="L721" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="M721" t="inlineStr">
-        <is>
-          <t>Etikettenband gerissen</t>
-        </is>
-      </c>
-      <c r="N721" t="inlineStr">
-        <is>
-          <t>Zu hohe Spannung</t>
-        </is>
-      </c>
-      <c r="O721" t="inlineStr">
-        <is>
-          <t>Produktionsstopp</t>
-        </is>
-      </c>
-      <c r="P721" t="inlineStr">
-        <is>
-          <t>Band neu einfädeln</t>
-        </is>
-      </c>
-    </row>
-    <row r="722">
-      <c r="A722" s="19" t="inlineStr">
-        <is>
-          <t>MAE</t>
-        </is>
-      </c>
-      <c r="B722" s="4" t="inlineStr">
-        <is>
-          <t>0025</t>
-        </is>
-      </c>
-      <c r="C722" s="44" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D722" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="E722" t="n">
-        <v>0</v>
-      </c>
-      <c r="G722" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="H722" s="53" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I722" t="inlineStr">
-        <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="J722" t="inlineStr">
-        <is>
-          <t>MAE0025 Störung Etikettenerfassung (Label zu kurz)</t>
-        </is>
-      </c>
-      <c r="K722" s="53" t="n"/>
-      <c r="L722" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="M722" t="inlineStr">
-        <is>
-          <t>Label zu kurz</t>
-        </is>
-      </c>
-      <c r="N722" t="inlineStr">
-        <is>
-          <t>Sensor falsch eingestellt</t>
-        </is>
-      </c>
-      <c r="O722" t="inlineStr">
-        <is>
-          <t>Produktionspause</t>
-        </is>
-      </c>
-      <c r="P722" t="inlineStr">
-        <is>
-          <t>Parameter prüfen, Sensor neu einmessen</t>
         </is>
       </c>
     </row>
@@ -49308,7 +49306,7 @@
       </c>
       <c r="B723" s="4" t="inlineStr">
         <is>
-          <t>0026</t>
+          <t>0024</t>
         </is>
       </c>
       <c r="C723" s="44" t="inlineStr">
@@ -49339,7 +49337,7 @@
       </c>
       <c r="J723" t="inlineStr">
         <is>
-          <t>MAE0026 Störung Etikettenerfassung (Label zu lang)</t>
+          <t>MAE0024 Etikettenbandriss</t>
         </is>
       </c>
       <c r="K723" s="53" t="n"/>
@@ -49350,22 +49348,22 @@
       </c>
       <c r="M723" t="inlineStr">
         <is>
-          <t>Label zu lang</t>
+          <t>Etikettenband gerissen</t>
         </is>
       </c>
       <c r="N723" t="inlineStr">
         <is>
-          <t>Sensor falsch eingestellt</t>
+          <t>Zu hohe Spannung</t>
         </is>
       </c>
       <c r="O723" t="inlineStr">
         <is>
-          <t>Produktionspause</t>
+          <t>Produktionsstopp</t>
         </is>
       </c>
       <c r="P723" t="inlineStr">
         <is>
-          <t>Parameter prüfen, Sensor neu einmessen</t>
+          <t>Band neu einfädeln</t>
         </is>
       </c>
     </row>
@@ -49377,7 +49375,7 @@
       </c>
       <c r="B724" s="4" t="inlineStr">
         <is>
-          <t>0027</t>
+          <t>0025</t>
         </is>
       </c>
       <c r="C724" s="44" t="inlineStr">
@@ -49408,7 +49406,7 @@
       </c>
       <c r="J724" t="inlineStr">
         <is>
-          <t>MAE0027 Störung Etikettenerfassung (Sensor prellt)</t>
+          <t>MAE0025 Störung Etikettenerfassung (Label zu kurz)</t>
         </is>
       </c>
       <c r="K724" s="53" t="n"/>
@@ -49419,164 +49417,164 @@
       </c>
       <c r="M724" t="inlineStr">
         <is>
+          <t>Label zu kurz</t>
+        </is>
+      </c>
+      <c r="N724" t="inlineStr">
+        <is>
+          <t>Sensor falsch eingestellt</t>
+        </is>
+      </c>
+      <c r="O724" t="inlineStr">
+        <is>
+          <t>Produktionspause</t>
+        </is>
+      </c>
+      <c r="P724" t="inlineStr">
+        <is>
+          <t>Parameter prüfen, Sensor neu einmessen</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" s="19" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="B725" s="4" t="inlineStr">
+        <is>
+          <t>0026</t>
+        </is>
+      </c>
+      <c r="C725" s="44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D725" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="E725" t="n">
+        <v>0</v>
+      </c>
+      <c r="G725" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="H725" s="53" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I725" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="J725" t="inlineStr">
+        <is>
+          <t>MAE0026 Störung Etikettenerfassung (Label zu lang)</t>
+        </is>
+      </c>
+      <c r="K725" s="53" t="n"/>
+      <c r="L725" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="M725" t="inlineStr">
+        <is>
+          <t>Label zu lang</t>
+        </is>
+      </c>
+      <c r="N725" t="inlineStr">
+        <is>
+          <t>Sensor falsch eingestellt</t>
+        </is>
+      </c>
+      <c r="O725" t="inlineStr">
+        <is>
+          <t>Produktionspause</t>
+        </is>
+      </c>
+      <c r="P725" t="inlineStr">
+        <is>
+          <t>Parameter prüfen, Sensor neu einmessen</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" s="19" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="B726" s="4" t="inlineStr">
+        <is>
+          <t>0027</t>
+        </is>
+      </c>
+      <c r="C726" s="44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D726" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="E726" t="n">
+        <v>0</v>
+      </c>
+      <c r="G726" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="H726" s="53" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I726" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="J726" t="inlineStr">
+        <is>
+          <t>MAE0027 Störung Etikettenerfassung (Sensor prellt)</t>
+        </is>
+      </c>
+      <c r="K726" s="53" t="n"/>
+      <c r="L726" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="M726" t="inlineStr">
+        <is>
           <t>Etikettenerfassungs-Sensor prellt</t>
         </is>
       </c>
-      <c r="N724" t="inlineStr">
+      <c r="N726" t="inlineStr">
         <is>
           <t>Sensor falsch eingestellt</t>
         </is>
       </c>
-      <c r="O724" t="inlineStr">
+      <c r="O726" t="inlineStr">
         <is>
           <t>Produktionspause</t>
         </is>
       </c>
-      <c r="P724" s="12" t="inlineStr">
+      <c r="P726" s="12" t="inlineStr">
         <is>
           <t>Sensor reinigen, neu einstellen, 
 Formatparameter prüfen</t>
         </is>
       </c>
     </row>
-    <row r="725">
-      <c r="A725" s="19" t="inlineStr">
-        <is>
-          <t>MAE</t>
-        </is>
-      </c>
-      <c r="B725" s="4" t="inlineStr">
-        <is>
-          <t>0028</t>
-        </is>
-      </c>
-      <c r="C725" s="44" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D725" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="E725" t="n">
-        <v>0</v>
-      </c>
-      <c r="G725" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="H725" s="53" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I725" t="inlineStr">
-        <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="J725" t="inlineStr">
-        <is>
-          <t>MAE0028 Störung Abwicklung (Tänzerarm blockiert)</t>
-        </is>
-      </c>
-      <c r="K725" s="53" t="n"/>
-      <c r="L725" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="M725" t="inlineStr">
-        <is>
-          <t>Tänzerarm der Abwicklung blockiert</t>
-        </is>
-      </c>
-      <c r="N725" t="inlineStr">
-        <is>
-          <t>Mechanische Blockade</t>
-        </is>
-      </c>
-      <c r="O725" t="inlineStr">
-        <is>
-          <t>Bandregelung gestört</t>
-        </is>
-      </c>
-      <c r="P725" t="inlineStr">
-        <is>
-          <t>Auf Blockade prüfen</t>
-        </is>
-      </c>
-    </row>
-    <row r="726">
-      <c r="A726" s="19" t="inlineStr">
-        <is>
-          <t>MAE</t>
-        </is>
-      </c>
-      <c r="B726" s="4" t="inlineStr">
-        <is>
-          <t>0029</t>
-        </is>
-      </c>
-      <c r="C726" s="44" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D726" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="E726" t="n">
-        <v>0</v>
-      </c>
-      <c r="G726" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="H726" s="53" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I726" t="inlineStr">
-        <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="J726" t="inlineStr">
-        <is>
-          <t>MAE0029 Störung Abwicklung (Tänzeram zu hoch)</t>
-        </is>
-      </c>
-      <c r="K726" s="53" t="n"/>
-      <c r="L726" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="M726" t="inlineStr">
-        <is>
-          <t>Tänzerarm der Abwicklung zu hoch</t>
-        </is>
-      </c>
-      <c r="N726" t="inlineStr">
-        <is>
-          <t>Spannung zu gering</t>
-        </is>
-      </c>
-      <c r="O726" t="inlineStr">
-        <is>
-          <t>Bandrissgefahr</t>
-        </is>
-      </c>
-      <c r="P726" t="inlineStr">
-        <is>
-          <t>Auf Blockade prüfen</t>
-        </is>
-      </c>
-    </row>
     <row r="727">
       <c r="A727" s="19" t="inlineStr">
         <is>
@@ -49585,7 +49583,7 @@
       </c>
       <c r="B727" s="4" t="inlineStr">
         <is>
-          <t>0030</t>
+          <t>0028</t>
         </is>
       </c>
       <c r="C727" s="44" t="inlineStr">
@@ -49616,7 +49614,7 @@
       </c>
       <c r="J727" t="inlineStr">
         <is>
-          <t>MAE0030 Störung Abwicklung (Tänzeram zu tief)</t>
+          <t>MAE0028 Störung Abwicklung (Tänzerarm blockiert)</t>
         </is>
       </c>
       <c r="K727" s="53" t="n"/>
@@ -49627,17 +49625,17 @@
       </c>
       <c r="M727" t="inlineStr">
         <is>
-          <t>Tänzerarm der Abwicklung zu tief</t>
+          <t>Tänzerarm der Abwicklung blockiert</t>
         </is>
       </c>
       <c r="N727" t="inlineStr">
         <is>
-          <t>Spannung zu hoch</t>
+          <t>Mechanische Blockade</t>
         </is>
       </c>
       <c r="O727" t="inlineStr">
         <is>
-          <t>Bandspannun nicht stuerbar</t>
+          <t>Bandregelung gestört</t>
         </is>
       </c>
       <c r="P727" t="inlineStr">
@@ -49654,7 +49652,7 @@
       </c>
       <c r="B728" s="4" t="inlineStr">
         <is>
-          <t>0031</t>
+          <t>0029</t>
         </is>
       </c>
       <c r="C728" s="44" t="inlineStr">
@@ -49685,7 +49683,7 @@
       </c>
       <c r="J728" t="inlineStr">
         <is>
-          <t>MAE0031 Störung Abwicklung (Falscher Kernadapter eingelegt)</t>
+          <t>MAE0029 Störung Abwicklung (Tänzeram zu hoch)</t>
         </is>
       </c>
       <c r="K728" s="53" t="n"/>
@@ -49696,22 +49694,22 @@
       </c>
       <c r="M728" t="inlineStr">
         <is>
-          <t>Falschen Kernadapter auf Abwicklung erkannt</t>
+          <t>Tänzerarm der Abwicklung zu hoch</t>
         </is>
       </c>
       <c r="N728" t="inlineStr">
         <is>
-          <t>Falscher Adapter eingesetzt</t>
+          <t>Spannung zu gering</t>
         </is>
       </c>
       <c r="O728" t="inlineStr">
         <is>
-          <t>Wickeln nicht möglich</t>
+          <t>Bandrissgefahr</t>
         </is>
       </c>
       <c r="P728" t="inlineStr">
         <is>
-          <t>Adapter tauschen</t>
+          <t>Auf Blockade prüfen</t>
         </is>
       </c>
     </row>
@@ -49723,7 +49721,7 @@
       </c>
       <c r="B729" s="4" t="inlineStr">
         <is>
-          <t>0032</t>
+          <t>0030</t>
         </is>
       </c>
       <c r="C729" s="44" t="inlineStr">
@@ -49754,7 +49752,7 @@
       </c>
       <c r="J729" t="inlineStr">
         <is>
-          <t>MAE0032 Störung Aufwicklung (Tänzerarm blockiert)</t>
+          <t>MAE0030 Störung Abwicklung (Tänzeram zu tief)</t>
         </is>
       </c>
       <c r="K729" s="53" t="n"/>
@@ -49765,17 +49763,17 @@
       </c>
       <c r="M729" t="inlineStr">
         <is>
-          <t>Tänzerarm der Aufwicklung blockiert</t>
+          <t>Tänzerarm der Abwicklung zu tief</t>
         </is>
       </c>
       <c r="N729" t="inlineStr">
         <is>
-          <t>Mechanische Blockade</t>
+          <t>Spannung zu hoch</t>
         </is>
       </c>
       <c r="O729" t="inlineStr">
         <is>
-          <t>Bandregelung gestört</t>
+          <t>Bandspannun nicht stuerbar</t>
         </is>
       </c>
       <c r="P729" t="inlineStr">
@@ -49792,7 +49790,7 @@
       </c>
       <c r="B730" s="4" t="inlineStr">
         <is>
-          <t>0033</t>
+          <t>0031</t>
         </is>
       </c>
       <c r="C730" s="44" t="inlineStr">
@@ -49823,7 +49821,7 @@
       </c>
       <c r="J730" t="inlineStr">
         <is>
-          <t>MAE0033 Störung Aufwicklung (Tänzeram zu hoch)</t>
+          <t>MAE0031 Störung Abwicklung (Falscher Kernadapter eingelegt)</t>
         </is>
       </c>
       <c r="K730" s="53" t="n"/>
@@ -49834,22 +49832,22 @@
       </c>
       <c r="M730" t="inlineStr">
         <is>
-          <t>Tänzerarm der Aufwicklung zu hoch</t>
+          <t>Falschen Kernadapter auf Abwicklung erkannt</t>
         </is>
       </c>
       <c r="N730" t="inlineStr">
         <is>
-          <t>Spannung zu gering</t>
+          <t>Falscher Adapter eingesetzt</t>
         </is>
       </c>
       <c r="O730" t="inlineStr">
         <is>
-          <t>Bandrissgefahr</t>
+          <t>Wickeln nicht möglich</t>
         </is>
       </c>
       <c r="P730" t="inlineStr">
         <is>
-          <t>Auf Blockade prüfen</t>
+          <t>Adapter tauschen</t>
         </is>
       </c>
     </row>
@@ -49861,7 +49859,7 @@
       </c>
       <c r="B731" s="4" t="inlineStr">
         <is>
-          <t>0034</t>
+          <t>0032</t>
         </is>
       </c>
       <c r="C731" s="44" t="inlineStr">
@@ -49892,7 +49890,7 @@
       </c>
       <c r="J731" t="inlineStr">
         <is>
-          <t>MAE0034 Störung Aufwicklung (Tänzeram zu tief)</t>
+          <t>MAE0032 Störung Aufwicklung (Tänzerarm blockiert)</t>
         </is>
       </c>
       <c r="K731" s="53" t="n"/>
@@ -49903,17 +49901,17 @@
       </c>
       <c r="M731" t="inlineStr">
         <is>
-          <t>Tänzerarm der Aufwicklung zu tief</t>
+          <t>Tänzerarm der Aufwicklung blockiert</t>
         </is>
       </c>
       <c r="N731" t="inlineStr">
         <is>
-          <t>Spannung zu hoch</t>
+          <t>Mechanische Blockade</t>
         </is>
       </c>
       <c r="O731" t="inlineStr">
         <is>
-          <t>Bandspannun nicht stuerbar</t>
+          <t>Bandregelung gestört</t>
         </is>
       </c>
       <c r="P731" t="inlineStr">
@@ -49930,7 +49928,7 @@
       </c>
       <c r="B732" s="4" t="inlineStr">
         <is>
-          <t>0035</t>
+          <t>0033</t>
         </is>
       </c>
       <c r="C732" s="44" t="inlineStr">
@@ -49961,7 +49959,7 @@
       </c>
       <c r="J732" t="inlineStr">
         <is>
-          <t>MAE0035 Störung Aufwicklung (Falscher Kernadapter eingelegt)</t>
+          <t>MAE0033 Störung Aufwicklung (Tänzeram zu hoch)</t>
         </is>
       </c>
       <c r="K732" s="53" t="n"/>
@@ -49972,22 +49970,22 @@
       </c>
       <c r="M732" t="inlineStr">
         <is>
-          <t>Falschen Kernadapter auf Aufwicklung erkannt</t>
+          <t>Tänzerarm der Aufwicklung zu hoch</t>
         </is>
       </c>
       <c r="N732" t="inlineStr">
         <is>
-          <t>Falscher Adapter eingesetzt</t>
+          <t>Spannung zu gering</t>
         </is>
       </c>
       <c r="O732" t="inlineStr">
         <is>
-          <t>Wickeln nicht möglich</t>
+          <t>Bandrissgefahr</t>
         </is>
       </c>
       <c r="P732" t="inlineStr">
         <is>
-          <t>Adapter tauschen</t>
+          <t>Auf Blockade prüfen</t>
         </is>
       </c>
     </row>
@@ -49999,7 +49997,7 @@
       </c>
       <c r="B733" s="4" t="inlineStr">
         <is>
-          <t>0036</t>
+          <t>0034</t>
         </is>
       </c>
       <c r="C733" s="44" t="inlineStr">
@@ -50030,7 +50028,7 @@
       </c>
       <c r="J733" t="inlineStr">
         <is>
-          <t>MAE0036 Wechsel zu Einrichtbetrieb fehlgeschlagen</t>
+          <t>MAE0034 Störung Aufwicklung (Tänzeram zu tief)</t>
         </is>
       </c>
       <c r="K733" s="53" t="n"/>
@@ -50041,17 +50039,17 @@
       </c>
       <c r="M733" t="inlineStr">
         <is>
-          <t>Einrichtbetrieb nicht erreichbar</t>
+          <t>Tänzerarm der Aufwicklung zu tief</t>
         </is>
       </c>
       <c r="N733" t="inlineStr">
         <is>
-          <t>Achsen nicht bereit oder Blockade im Fahrtweg</t>
+          <t>Spannung zu hoch</t>
         </is>
       </c>
       <c r="O733" t="inlineStr">
         <is>
-          <t>Produktionsstopp</t>
+          <t>Bandspannun nicht stuerbar</t>
         </is>
       </c>
       <c r="P733" t="inlineStr">
@@ -50068,7 +50066,7 @@
       </c>
       <c r="B734" s="4" t="inlineStr">
         <is>
-          <t>0037</t>
+          <t>0035</t>
         </is>
       </c>
       <c r="C734" s="44" t="inlineStr">
@@ -50099,7 +50097,7 @@
       </c>
       <c r="J734" t="inlineStr">
         <is>
-          <t>MAE0037 Wechsel zu Produktionsbetrieb fehlgeschlagen</t>
+          <t>MAE0035 Störung Aufwicklung (Falscher Kernadapter eingelegt)</t>
         </is>
       </c>
       <c r="K734" s="53" t="n"/>
@@ -50110,22 +50108,22 @@
       </c>
       <c r="M734" t="inlineStr">
         <is>
-          <t>Produktionsbetrieb nicht erreichbar</t>
+          <t>Falschen Kernadapter auf Aufwicklung erkannt</t>
         </is>
       </c>
       <c r="N734" t="inlineStr">
         <is>
-          <t>Achsen nicht bereit oder Blockade im Fahrtweg</t>
+          <t>Falscher Adapter eingesetzt</t>
         </is>
       </c>
       <c r="O734" t="inlineStr">
         <is>
-          <t>Produktion startet nicht</t>
+          <t>Wickeln nicht möglich</t>
         </is>
       </c>
       <c r="P734" t="inlineStr">
         <is>
-          <t>Auf Blockade prüfen</t>
+          <t>Adapter tauschen</t>
         </is>
       </c>
     </row>
@@ -50137,7 +50135,7 @@
       </c>
       <c r="B735" s="4" t="inlineStr">
         <is>
-          <t>0038</t>
+          <t>0036</t>
         </is>
       </c>
       <c r="C735" s="44" t="inlineStr">
@@ -50168,7 +50166,7 @@
       </c>
       <c r="J735" t="inlineStr">
         <is>
-          <t>MAE0038 Wechsel zu Pause Fehlgeschlagen</t>
+          <t>MAE0036 Wechsel zu Einrichtbetrieb fehlgeschlagen</t>
         </is>
       </c>
       <c r="K735" s="53" t="n"/>
@@ -50179,12 +50177,17 @@
       </c>
       <c r="M735" t="inlineStr">
         <is>
-          <t>Pause nicht erreichbar</t>
+          <t>Einrichtbetrieb nicht erreichbar</t>
+        </is>
+      </c>
+      <c r="N735" t="inlineStr">
+        <is>
+          <t>Achsen nicht bereit oder Blockade im Fahrtweg</t>
         </is>
       </c>
       <c r="O735" t="inlineStr">
         <is>
-          <t>Produktionspause</t>
+          <t>Produktionsstopp</t>
         </is>
       </c>
       <c r="P735" t="inlineStr">
@@ -50201,7 +50204,7 @@
       </c>
       <c r="B736" s="4" t="inlineStr">
         <is>
-          <t>0039</t>
+          <t>0037</t>
         </is>
       </c>
       <c r="C736" s="44" t="inlineStr">
@@ -50232,7 +50235,7 @@
       </c>
       <c r="J736" t="inlineStr">
         <is>
-          <t>MAE0039 Wechsel zu Produktionsstop fehlgeschlagen</t>
+          <t>MAE0037 Wechsel zu Produktionsbetrieb fehlgeschlagen</t>
         </is>
       </c>
       <c r="K736" s="53" t="n"/>
@@ -50243,12 +50246,17 @@
       </c>
       <c r="M736" t="inlineStr">
         <is>
-          <t>Produktionsstopp nicht möglich</t>
+          <t>Produktionsbetrieb nicht erreichbar</t>
+        </is>
+      </c>
+      <c r="N736" t="inlineStr">
+        <is>
+          <t>Achsen nicht bereit oder Blockade im Fahrtweg</t>
         </is>
       </c>
       <c r="O736" t="inlineStr">
         <is>
-          <t>Produktionspause</t>
+          <t>Produktion startet nicht</t>
         </is>
       </c>
       <c r="P736" t="inlineStr">
@@ -50265,7 +50273,7 @@
       </c>
       <c r="B737" s="4" t="inlineStr">
         <is>
-          <t>0040</t>
+          <t>0038</t>
         </is>
       </c>
       <c r="C737" s="44" t="inlineStr">
@@ -50296,7 +50304,7 @@
       </c>
       <c r="J737" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAE0040 Wechsel zu Rückspulbetrieb fehlgeschlagen </t>
+          <t>MAE0038 Wechsel zu Pause Fehlgeschlagen</t>
         </is>
       </c>
       <c r="K737" s="53" t="n"/>
@@ -50307,12 +50315,12 @@
       </c>
       <c r="M737" t="inlineStr">
         <is>
-          <t>Rückspulbetrieb nicht möglich</t>
+          <t>Pause nicht erreichbar</t>
         </is>
       </c>
       <c r="O737" t="inlineStr">
         <is>
-          <t>Rückspulen blockiert</t>
+          <t>Produktionspause</t>
         </is>
       </c>
       <c r="P737" t="inlineStr">
@@ -50329,7 +50337,7 @@
       </c>
       <c r="B738" s="4" t="inlineStr">
         <is>
-          <t>0041</t>
+          <t>0039</t>
         </is>
       </c>
       <c r="C738" s="44" t="inlineStr">
@@ -50360,7 +50368,7 @@
       </c>
       <c r="J738" t="inlineStr">
         <is>
-          <t>MAE0041 Wechsel zu Etikettenentnahme</t>
+          <t>MAE0039 Wechsel zu Produktionsstop fehlgeschlagen</t>
         </is>
       </c>
       <c r="K738" s="53" t="n"/>
@@ -50371,7 +50379,7 @@
       </c>
       <c r="M738" t="inlineStr">
         <is>
-          <t>Wechsel zu Etikettenentnahme nicht möglich</t>
+          <t>Produktionsstopp nicht möglich</t>
         </is>
       </c>
       <c r="O738" t="inlineStr">
@@ -50393,7 +50401,7 @@
       </c>
       <c r="B739" s="4" t="inlineStr">
         <is>
-          <t>0042</t>
+          <t>0040</t>
         </is>
       </c>
       <c r="C739" s="44" t="inlineStr">
@@ -50424,7 +50432,7 @@
       </c>
       <c r="J739" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAE0042 Wechsel zu Spleissen fehlgeschlagen </t>
+          <t xml:space="preserve">MAE0040 Wechsel zu Rückspulbetrieb fehlgeschlagen </t>
         </is>
       </c>
       <c r="K739" s="53" t="n"/>
@@ -50435,12 +50443,12 @@
       </c>
       <c r="M739" t="inlineStr">
         <is>
-          <t>Spleissbetrieb nicht möglich</t>
+          <t>Rückspulbetrieb nicht möglich</t>
         </is>
       </c>
       <c r="O739" t="inlineStr">
         <is>
-          <t>Spleissen blockiert</t>
+          <t>Rückspulen blockiert</t>
         </is>
       </c>
       <c r="P739" t="inlineStr">
@@ -50457,7 +50465,7 @@
       </c>
       <c r="B740" s="4" t="inlineStr">
         <is>
-          <t>0043</t>
+          <t>0041</t>
         </is>
       </c>
       <c r="C740" s="44" t="inlineStr">
@@ -50488,7 +50496,7 @@
       </c>
       <c r="J740" t="inlineStr">
         <is>
-          <t>MAE0043 Wechsel zu Synchronisieren fehlgeschlagen</t>
+          <t>MAE0041 Wechsel zu Etikettenentnahme</t>
         </is>
       </c>
       <c r="K740" s="53" t="n"/>
@@ -50499,17 +50507,12 @@
       </c>
       <c r="M740" t="inlineStr">
         <is>
-          <t>Synchronisieren fehlgeschlagen</t>
-        </is>
-      </c>
-      <c r="N740" t="inlineStr">
-        <is>
-          <t>Achsen nicht bereit oder Blockade im Fahrtweg</t>
+          <t>Wechsel zu Etikettenentnahme nicht möglich</t>
         </is>
       </c>
       <c r="O740" t="inlineStr">
         <is>
-          <t>Produktionsstopp</t>
+          <t>Produktionspause</t>
         </is>
       </c>
       <c r="P740" t="inlineStr">
@@ -50526,7 +50529,7 @@
       </c>
       <c r="B741" s="4" t="inlineStr">
         <is>
-          <t>0044</t>
+          <t>0042</t>
         </is>
       </c>
       <c r="C741" s="44" t="inlineStr">
@@ -50557,7 +50560,7 @@
       </c>
       <c r="J741" t="inlineStr">
         <is>
-          <t>MAE0044 Wechsel zu Produktion abgeschlossen fehlgeschlagen</t>
+          <t xml:space="preserve">MAE0042 Wechsel zu Spleissen fehlgeschlagen </t>
         </is>
       </c>
       <c r="K741" s="53" t="n"/>
@@ -50568,12 +50571,12 @@
       </c>
       <c r="M741" t="inlineStr">
         <is>
-          <t>Produktion abgeschlossen fehlgeschlagen</t>
+          <t>Spleissbetrieb nicht möglich</t>
         </is>
       </c>
       <c r="O741" t="inlineStr">
         <is>
-          <t>Produktionspause</t>
+          <t>Spleissen blockiert</t>
         </is>
       </c>
       <c r="P741" t="inlineStr">
@@ -50590,7 +50593,7 @@
       </c>
       <c r="B742" s="4" t="inlineStr">
         <is>
-          <t>0045</t>
+          <t>0043</t>
         </is>
       </c>
       <c r="C742" s="44" t="inlineStr">
@@ -50621,7 +50624,7 @@
       </c>
       <c r="J742" t="inlineStr">
         <is>
-          <t>MAE0045 Störung während Rückspulung</t>
+          <t>MAE0043 Wechsel zu Synchronisieren fehlgeschlagen</t>
         </is>
       </c>
       <c r="K742" s="53" t="n"/>
@@ -50632,20 +50635,153 @@
       </c>
       <c r="M742" t="inlineStr">
         <is>
+          <t>Synchronisieren fehlgeschlagen</t>
+        </is>
+      </c>
+      <c r="N742" t="inlineStr">
+        <is>
+          <t>Achsen nicht bereit oder Blockade im Fahrtweg</t>
+        </is>
+      </c>
+      <c r="O742" t="inlineStr">
+        <is>
+          <t>Produktionsstopp</t>
+        </is>
+      </c>
+      <c r="P742" t="inlineStr">
+        <is>
+          <t>Auf Blockade prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" s="19" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="B743" s="4" t="inlineStr">
+        <is>
+          <t>0044</t>
+        </is>
+      </c>
+      <c r="C743" s="44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D743" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="E743" t="n">
+        <v>0</v>
+      </c>
+      <c r="G743" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="H743" s="53" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I743" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="J743" t="inlineStr">
+        <is>
+          <t>MAE0044 Wechsel zu Produktion abgeschlossen fehlgeschlagen</t>
+        </is>
+      </c>
+      <c r="K743" s="53" t="n"/>
+      <c r="L743" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="M743" t="inlineStr">
+        <is>
+          <t>Produktion abgeschlossen fehlgeschlagen</t>
+        </is>
+      </c>
+      <c r="O743" t="inlineStr">
+        <is>
+          <t>Produktionspause</t>
+        </is>
+      </c>
+      <c r="P743" t="inlineStr">
+        <is>
+          <t>Auf Blockade prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" s="19" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="B744" s="4" t="inlineStr">
+        <is>
+          <t>0045</t>
+        </is>
+      </c>
+      <c r="C744" s="44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D744" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="E744" t="n">
+        <v>0</v>
+      </c>
+      <c r="G744" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="H744" s="53" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I744" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="J744" t="inlineStr">
+        <is>
+          <t>MAE0045 Störung während Rückspulung</t>
+        </is>
+      </c>
+      <c r="K744" s="53" t="n"/>
+      <c r="L744" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="M744" t="inlineStr">
+        <is>
           <t>Fehler während Rückspulung</t>
         </is>
       </c>
-      <c r="N742" t="inlineStr">
+      <c r="N744" t="inlineStr">
         <is>
           <t>Blockade oder Encoder-Fehler</t>
         </is>
       </c>
-      <c r="O742" t="inlineStr">
+      <c r="O744" t="inlineStr">
         <is>
           <t>Rückspulung abgebrochen</t>
         </is>
       </c>
-      <c r="P742" t="inlineStr">
+      <c r="P744" t="inlineStr">
         <is>
           <t>Encoder und Etikettenlauf prüfen</t>
         </is>
@@ -50940,22 +51076,22 @@
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
-    <TaxCatchAll xmlns="d728571b-78ef-4dbd-85be-d4d1cda44c95" xsi:nil="true"/>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="9c94746f-923d-44d4-92c8-8aca0d670c40">
       <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d728571b-78ef-4dbd-85be-d4d1cda44c95" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACC13BB1-D6E9-4F18-BDE9-4832F5BECDE6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E0B9B61-108C-4949-AEC7-3ECD2EA73843}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D15969F1-8C9A-4461-861C-965F23471A22}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FC2439E-2A0E-4F7F-8387-6691388526F0}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EDCA1D26-6613-42F0-93E8-BCBE5FE7E935}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{161DDA0F-7F0A-4D3B-A8ED-EB5198B68FF3}"/>
 </file>
</xml_diff>